<commit_message>
categorized glossaries, morphotype lookup fixes
</commit_message>
<xml_diff>
--- a/app_kit/tests/TESTS_ROOT/xlsx_for_testing/Glossary/valid/Glossary.xlsx
+++ b/app_kit/tests/TESTS_ROOT/xlsx_for_testing/Glossary/valid/Glossary.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Glossary" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">Term</t>
   </si>
@@ -32,6 +32,9 @@
     <t xml:space="preserve">Definition</t>
   </si>
   <si>
+    <t xml:space="preserve">Category (optional)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bark</t>
   </si>
   <si>
@@ -51,6 +54,15 @@
   </si>
   <si>
     <t xml:space="preserve">underground water that moves downward under the influence of gravity  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categorized term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defintion of a categorized entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">category</t>
   </si>
 </sst>
 </file>
@@ -145,7 +157,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -164,6 +176,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -355,7 +371,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="63.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="4" style="2" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="25.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="5" style="2" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -368,34 +385,48 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="AMI1" s="2"/>
       <c r="AMJ1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>